<commit_message>
chore: update KPI targets (cost/revenue/ROAS)
- 네이버브랜드스토어: cost 450,000,000 -> 315,572,962 / revenue 1,503,690,564 -> 1,745,384,267 / ROAS 3.34 -> 5.53
- 쿠팡: cost 450,000,000 -> 331,145,922 / revenue 4,705,242,873 -> 3,810,119,469 / ROAS 10.46 -> 11.51
- othermall: cost 45,100,000 -> 46,194,206 / revenue 49,541,667 -> 108,884,478 / ROAS 1.10 -> 2.36

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/KPI.xlsx
+++ b/KPI.xlsx
@@ -1,107 +1,49 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MADUP\주식회사매드업 Dropbox\광고사업부\4. 광고주\샤크닌자\바이브코딩\02. 데일리리포트 대시보드\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B0BB68F2-121B-4142-B2B5-0A0CFC74828D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="43080" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D77A43E8-DBF1-4515-988C-51BEECCED695}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="43080" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
-  <si>
-    <t>채널</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>목표 비용</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>목표 매출</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>네이버브랜드스토어</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>쿠팡</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>othermall</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>목표 ROAS</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="6" formatCode="&quot;₩&quot;#,##0;[Red]\-&quot;₩&quot;#,##0"/>
+    <numFmt numFmtId="164" formatCode="&quot;₩&quot;#,##0;[Red]\-&quot;₩&quot;#,##0"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="2"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="맑은 고딕"/>
-      <family val="2"/>
-      <charset val="129"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="2"/>
       <sz val="8"/>
-      <name val="맑은 고딕"/>
-      <family val="2"/>
-      <charset val="129"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -117,34 +59,97 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="6" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -464,73 +469,90 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5521F7AB-CCC3-4EF9-AE61-3EF66AFC6025}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16.9"/>
   <cols>
-    <col min="1" max="1" width="17.75" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.625" bestFit="1" customWidth="1"/>
+    <col width="17.75" bestFit="1" customWidth="1" style="3" min="1" max="1"/>
+    <col width="12.125" bestFit="1" customWidth="1" style="3" min="2" max="2"/>
+    <col width="13.625" bestFit="1" customWidth="1" style="3" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.6">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>6</v>
+    <row r="1">
+      <c r="A1" s="0" t="inlineStr">
+        <is>
+          <t>채널</t>
+        </is>
+      </c>
+      <c r="B1" s="0" t="inlineStr">
+        <is>
+          <t>목표 비용</t>
+        </is>
+      </c>
+      <c r="C1" s="0" t="inlineStr">
+        <is>
+          <t>목표 매출</t>
+        </is>
+      </c>
+      <c r="D1" s="0" t="inlineStr">
+        <is>
+          <t>목표 ROAS</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.6">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="1">
-        <v>450000000</v>
-      </c>
-      <c r="C2" s="1">
-        <v>1503690564</v>
-      </c>
-      <c r="D2" s="2">
-        <v>3.34</v>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>네이버브랜드스토어</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n">
+        <v>315572962</v>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>1745384267</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>5.53</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.6">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="1">
-        <v>450000000</v>
-      </c>
-      <c r="C3" s="1">
-        <v>4705242873</v>
-      </c>
-      <c r="D3" s="2">
-        <v>10.46</v>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>쿠팡</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>331145922</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>3810119469</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>11.51</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.6">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="1">
-        <v>45100000</v>
-      </c>
-      <c r="C4" s="1">
-        <v>49541667</v>
-      </c>
-      <c r="D4" s="2">
-        <v>1.1000000000000001</v>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>othermall</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>46194206</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>108884478</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>2.36</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: update KPI targets and split D2C into its own KPI card
KPI.xlsx 의 채널별 목표를 최신 기준으로 갱신하고, D2C 를 별도 채널로 추가한다.

- 네이버브랜드스토어: 비용 277,165,236 / 매출 1,278,665,072 / ROAS 4.61
- 쿠팡: 비용 461,942,060 / 매출 8,122,614,700 / ROAS 17.58
- othermall: 비용 61,592,274 / 매출 200,309,118 / ROAS 3.25
- D2C(신규): 비용 65,398,068 / 매출 196,163,375 / ROAS 3.00

D2C 는 그동안 othermall 에 합산돼 있었다. 별도 KPI 로 잡으면서
othermall 집계에서 D2C 를 빼 이중 집계를 막는다.

KPI 카드는 st.columns(3) 고정 대신 채널 수만큼 만들도록 바꿔서,
앞으로 KPI.xlsx 에 행을 추가/삭제해도 코드를 고칠 필요가 없다.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/KPI.xlsx
+++ b/KPI.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.9"/>
   <cols>
     <col width="17.75" bestFit="1" customWidth="1" style="3" min="1" max="1"/>
@@ -511,13 +511,13 @@
         </is>
       </c>
       <c r="B2" s="4" t="n">
-        <v>315572962</v>
+        <v>277165236</v>
       </c>
       <c r="C2" s="4" t="n">
-        <v>1745384267</v>
+        <v>1278665072</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>5.53</v>
+        <v>4.61</v>
       </c>
     </row>
     <row r="3">
@@ -527,13 +527,13 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>331145922</v>
+        <v>461942060</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>3810119469</v>
+        <v>8122614700</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>11.51</v>
+        <v>17.58</v>
       </c>
     </row>
     <row r="4">
@@ -543,13 +543,29 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>46194206</v>
+        <v>61592274</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>108884478</v>
+        <v>200309118</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>2.36</v>
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>D2C</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>65398068</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>196163375</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>